<commit_message>
docs(governance): preserve LP-003 V1 deferral (#41)
</commit_message>
<xml_diff>
--- a/Requirements/Babysteps_Platform_Requirements_FINAL_v65.xlsx
+++ b/Requirements/Babysteps_Platform_Requirements_FINAL_v65.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Workbook_Guide" sheetId="1" r:id="R495064ef50bc410b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="2" r:id="Rf36ba7383e504a2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Frozen_Requirements" sheetId="3" r:id="Rbbdd9a1390074d49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_v64_Requirements" sheetId="4" r:id="R4e0ac6683b3146a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Decision_Log" sheetId="5" r:id="R0c296936b1c143b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Acceptance_Tests_v64" sheetId="6" r:id="R94d2f4b63d4f4fe8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Requirement_Roadmap" sheetId="7" r:id="Rb0041977145c4dd4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_BB17_Superseded" sheetId="8" r:id="Re5cfac4045a24553"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Official_Sources" sheetId="9" r:id="R4fcd192fb72a4e30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_Workbook_Guide" sheetId="1" r:id="Rff09f69df2404db8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Dashboard" sheetId="2" r:id="R4553dd95f0614b9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Frozen_Requirements" sheetId="3" r:id="R6a9210a4b2e3435b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_v64_Requirements" sheetId="4" r:id="R8e7cbcbe3c834a8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Decision_Log" sheetId="5" r:id="R47152f31b3164bc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Acceptance_Tests_v64" sheetId="6" r:id="Rde919ff06ac9402f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Requirement_Roadmap" sheetId="7" r:id="R823d628964724999"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_BB17_Superseded" sheetId="8" r:id="Rbcbe28b679fd417a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Official_Sources" sheetId="9" r:id="R1b1da17ca4164abe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26,7 +26,7 @@
     <x:numFmt numFmtId="201" formatCode="yyyy-mm-dd hh:mm"/>
     <x:numFmt numFmtId="202" formatCode="0%"/>
   </x:numFmts>
-  <x:fonts count="5">
+  <x:fonts count="6">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -55,8 +55,14 @@
       <x:color rgb="FF6B21A8"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF7F6000"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -98,6 +104,16 @@
         <x:fgColor rgb="FF1F5D8D"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE7F5EA"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -106,7 +122,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="51">
+  <x:cellXfs count="55">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -210,6 +226,18 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -471,7 +499,7 @@
         <x:v>Active platform requirements</x:v>
       </x:c>
       <x:c r="B6" s="22" t="n">
-        <x:v>67</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="C6" s="22" t="str">
         <x:v>Final</x:v>
@@ -483,7 +511,7 @@
         <x:v>Frozen active requirements</x:v>
       </x:c>
       <x:c r="B7" s="22" t="n">
-        <x:v>67</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="C7" s="22" t="str">
         <x:v>Final</x:v>
@@ -602,7 +630,7 @@
         <x:v>Frozen active requirements</x:v>
       </x:c>
       <x:c r="B4" t="n">
-        <x:v>67</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="D4" t="str">
         <x:v>Identity and authentication</x:v>
@@ -631,10 +659,10 @@
         <x:v>Learner profiles and guardians</x:v>
       </x:c>
       <x:c r="E5" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F5" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G5" t="n">
         <x:v>0</x:v>
@@ -648,7 +676,7 @@
         <x:v>Active platform requirements</x:v>
       </x:c>
       <x:c r="B6" t="n">
-        <x:v>67</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="D6" t="str">
         <x:v>App registry</x:v>
@@ -695,7 +723,7 @@
         <x:v>Must Haves frozen</x:v>
       </x:c>
       <x:c r="B8" t="n">
-        <x:v>67</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="D8" t="str">
         <x:v>Authorization</x:v>
@@ -741,7 +769,7 @@
         <x:v>Codex Ready / frozen baseline</x:v>
       </x:c>
       <x:c r="B10" t="n">
-        <x:v>67</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="D10" t="str">
         <x:v>Billing and subscriptions</x:v>
@@ -833,7 +861,7 @@
         <x:v>Deferred requirements (outside active set)</x:v>
       </x:c>
       <x:c r="B14" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D14" t="str">
         <x:v>Engagement and gamification</x:v>
@@ -992,7 +1020,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="4" t="str">
-        <x:v>Frozen Requirements Register — 67 of 67 Active Platform Requirements</x:v>
+        <x:v>Requirements Register — 66 Active Platform Requirements + 1 Confirmed Deferral</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
       <x:c r="C1" s="4"/>
@@ -1195,19 +1223,19 @@
         <x:v>Learner Profiles &amp; Guardians</x:v>
       </x:c>
       <x:c r="D10" s="22" t="str">
-        <x:v>Carried forward unchanged from v63 authoritative frozen specification</x:v>
+        <x:v>Additional guardian access remains outside Version 1 under DEC-SCOPE-005; owner_parent_id is the sole learner-management authority.</x:v>
       </x:c>
       <x:c r="E10" s="22" t="str">
-        <x:v>Must Have</x:v>
-      </x:c>
-      <x:c r="F10" s="31" t="str">
-        <x:v>Approved</x:v>
-      </x:c>
-      <x:c r="G10" s="31" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Should Have</x:v>
+      </x:c>
+      <x:c r="F10" s="52" t="str">
+        <x:v>Deferred</x:v>
+      </x:c>
+      <x:c r="G10" s="52" t="str">
+        <x:v>No</x:v>
       </x:c>
       <x:c r="H10" s="22" t="str">
-        <x:v>v63 carried forward</x:v>
+        <x:v>v63 deferral confirmed in v65</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -3575,6 +3603,26 @@
         <x:v>Each consumer app creates app-specific UI/content/domain interactions; shared platform behavior is inherited from the common container.</x:v>
       </x:c>
     </x:row>
+    <x:row r="17" ht="58" customHeight="1">
+      <x:c r="A17" s="22" t="str">
+        <x:v>DEC-SCOPE-005</x:v>
+      </x:c>
+      <x:c r="B17" s="22" t="str">
+        <x:v>LP-003</x:v>
+      </x:c>
+      <x:c r="C17" s="22" t="str">
+        <x:v>Preserve the v63 deferral of additional guardian access outside Version 1. Exactly one owning parent manages each learner through owner_parent_id; no guardian invitation, sharing, household, or second-adult management surface is authorized.</x:v>
+      </x:c>
+      <x:c r="D17" s="54" t="str">
+        <x:v>Frozen</x:v>
+      </x:c>
+      <x:c r="E17" s="22" t="str">
+        <x:v>2026-08-24</x:v>
+      </x:c>
+      <x:c r="F17" s="22" t="str">
+        <x:v>Confirms Option A from GitHub issue #41. LP-003 is excluded from active V1 readiness counts unless a future approved specification explicitly supersedes this decision.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>
@@ -4240,10 +4288,10 @@
         <x:v>Learner profiles and guardians</x:v>
       </x:c>
       <x:c r="E5" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F5" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="G5" t="n">
         <x:v>0</x:v>

</xml_diff>